<commit_message>
Update JMDC and Optum DOD smoking concepts
</commit_message>
<xml_diff>
--- a/docs/JMDC/Vocab Updates/Annual_Health_Checkup_Mapping.xlsx
+++ b/docs/JMDC/Vocab Updates/Annual_Health_Checkup_Mapping.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10209"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10125"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/eburrow3/Documents/Git/ETL-LambdaBuilder/docs/JMDC/Vocab Updates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{556CACD1-2337-0D4D-B0B5-F5118681B7D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BB897CD-F8EF-234B-85B3-E043EF150575}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="42860" windowHeight="21020" tabRatio="856" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -544,10 +544,6 @@
     <t>Fundus_examination(Keith-Wagener_classification)</t>
   </si>
   <si>
-    <t>1=4298794
-2=4222303</t>
-  </si>
-  <si>
     <t>1=Smoker
 2=Non-smoker</t>
   </si>
@@ -605,11 +601,6 @@
   </si>
   <si>
     <t>smoking_habit_after_apr_24</t>
-  </si>
-  <si>
-    <t>1=4298794
-2=4310250
-3=4222303</t>
   </si>
   <si>
     <t>1=Smoker
@@ -743,6 +734,16 @@
     <t>1=4288153 
 2=765707
 3=763696</t>
+  </si>
+  <si>
+    <t>1=903657
+2=903651</t>
+  </si>
+  <si>
+    <t>1=903657	
+2=903651
+2=1340204
+3=903651</t>
   </si>
 </sst>
 </file>
@@ -1049,7 +1050,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1091,6 +1092,12 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2148,22 +2155,22 @@
     </row>
     <row r="29" spans="1:10" ht="105">
       <c r="A29" s="13" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B29" s="13" t="s">
+        <v>141</v>
+      </c>
+      <c r="C29" s="13" t="s">
         <v>142</v>
-      </c>
-      <c r="C29" s="13" t="s">
-        <v>143</v>
       </c>
       <c r="D29" s="13" t="s">
         <v>100</v>
       </c>
       <c r="E29" s="14" t="s">
+        <v>177</v>
+      </c>
+      <c r="F29" s="14" t="s">
         <v>132</v>
-      </c>
-      <c r="F29" s="14" t="s">
-        <v>133</v>
       </c>
       <c r="G29" s="14"/>
       <c r="H29" s="14"/>
@@ -2174,239 +2181,239 @@
     </row>
     <row r="30" spans="1:10" ht="135">
       <c r="A30" s="13" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B30" s="13" t="s">
+        <v>143</v>
+      </c>
+      <c r="C30" s="13" t="s">
         <v>144</v>
-      </c>
-      <c r="C30" s="13" t="s">
-        <v>145</v>
       </c>
       <c r="D30" s="13" t="s">
         <v>100</v>
       </c>
       <c r="E30" s="14" t="s">
-        <v>148</v>
+        <v>178</v>
       </c>
       <c r="F30" s="14" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="G30" s="14"/>
       <c r="H30" s="14"/>
       <c r="I30" s="14"/>
       <c r="J30" s="14" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" ht="45">
+      <c r="A31" s="15" t="s">
+        <v>149</v>
+      </c>
+      <c r="B31" s="15" t="s">
         <v>150</v>
       </c>
-    </row>
-    <row r="31" spans="1:10" ht="45">
-      <c r="A31" s="13" t="s">
+      <c r="C31" s="15" t="s">
         <v>151</v>
       </c>
-      <c r="B31" s="13" t="s">
+      <c r="D31" s="15" t="s">
+        <v>100</v>
+      </c>
+      <c r="E31" s="16"/>
+      <c r="F31" s="16"/>
+      <c r="G31" s="16"/>
+      <c r="H31" s="16"/>
+      <c r="I31" s="16"/>
+      <c r="J31" s="16" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" ht="45">
+      <c r="A32" s="15" t="s">
         <v>152</v>
       </c>
-      <c r="C31" s="13" t="s">
+      <c r="B32" s="15" t="s">
         <v>153</v>
       </c>
-      <c r="D31" s="13" t="s">
+      <c r="C32" s="15" t="s">
+        <v>142</v>
+      </c>
+      <c r="D32" s="15" t="s">
         <v>100</v>
       </c>
-      <c r="E31" s="14"/>
-      <c r="F31" s="14"/>
-      <c r="G31" s="14"/>
-      <c r="H31" s="14"/>
-      <c r="I31" s="14"/>
-      <c r="J31" s="14" t="s">
+      <c r="E32" s="16"/>
+      <c r="F32" s="16"/>
+      <c r="G32" s="16"/>
+      <c r="H32" s="16"/>
+      <c r="I32" s="16" t="s">
+        <v>89</v>
+      </c>
+      <c r="J32" s="16" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" ht="75">
+      <c r="A33" s="15" t="s">
+        <v>154</v>
+      </c>
+      <c r="B33" s="15" t="s">
+        <v>155</v>
+      </c>
+      <c r="C33" s="15" t="s">
+        <v>142</v>
+      </c>
+      <c r="D33" s="15" t="s">
+        <v>100</v>
+      </c>
+      <c r="E33" s="16"/>
+      <c r="F33" s="16"/>
+      <c r="G33" s="16"/>
+      <c r="H33" s="16"/>
+      <c r="I33" s="16" t="s">
+        <v>89</v>
+      </c>
+      <c r="J33" s="16" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" ht="60">
+      <c r="A34" s="15" t="s">
+        <v>156</v>
+      </c>
+      <c r="B34" s="15" t="s">
+        <v>157</v>
+      </c>
+      <c r="C34" s="15" t="s">
+        <v>158</v>
+      </c>
+      <c r="D34" s="15" t="s">
+        <v>100</v>
+      </c>
+      <c r="E34" s="16"/>
+      <c r="F34" s="16"/>
+      <c r="G34" s="16"/>
+      <c r="H34" s="16"/>
+      <c r="I34" s="16" t="s">
+        <v>176</v>
+      </c>
+      <c r="J34" s="16" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10" ht="30">
+      <c r="A35" s="15" t="s">
+        <v>159</v>
+      </c>
+      <c r="B35" s="15" t="s">
+        <v>160</v>
+      </c>
+      <c r="C35" s="15" t="s">
+        <v>142</v>
+      </c>
+      <c r="D35" s="15" t="s">
+        <v>100</v>
+      </c>
+      <c r="E35" s="16"/>
+      <c r="F35" s="16"/>
+      <c r="G35" s="16"/>
+      <c r="H35" s="16"/>
+      <c r="I35" s="16" t="s">
+        <v>89</v>
+      </c>
+      <c r="J35" s="16" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="36" spans="1:10" ht="60">
+      <c r="A36" s="15" t="s">
+        <v>163</v>
+      </c>
+      <c r="B36" s="15" t="s">
         <v>164</v>
       </c>
-    </row>
-    <row r="32" spans="1:10" ht="45">
-      <c r="A32" s="13" t="s">
-        <v>154</v>
-      </c>
-      <c r="B32" s="13" t="s">
-        <v>155</v>
-      </c>
-      <c r="C32" s="13" t="s">
-        <v>143</v>
-      </c>
-      <c r="D32" s="13" t="s">
+      <c r="C36" s="15" t="s">
+        <v>158</v>
+      </c>
+      <c r="D36" s="15" t="s">
         <v>100</v>
       </c>
-      <c r="E32" s="14"/>
-      <c r="F32" s="14"/>
-      <c r="G32" s="14"/>
-      <c r="H32" s="14"/>
-      <c r="I32" s="14" t="s">
-        <v>89</v>
-      </c>
-      <c r="J32" s="14" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="33" spans="1:10" ht="75">
-      <c r="A33" s="13" t="s">
-        <v>156</v>
-      </c>
-      <c r="B33" s="13" t="s">
-        <v>157</v>
-      </c>
-      <c r="C33" s="13" t="s">
-        <v>143</v>
-      </c>
-      <c r="D33" s="13" t="s">
+      <c r="E36" s="16"/>
+      <c r="F36" s="16"/>
+      <c r="G36" s="16"/>
+      <c r="H36" s="16"/>
+      <c r="I36" s="16" t="s">
+        <v>176</v>
+      </c>
+      <c r="J36" s="16" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10" ht="60">
+      <c r="A37" s="15" t="s">
+        <v>165</v>
+      </c>
+      <c r="B37" s="15" t="s">
+        <v>166</v>
+      </c>
+      <c r="C37" s="15" t="s">
+        <v>167</v>
+      </c>
+      <c r="D37" s="15" t="s">
         <v>100</v>
       </c>
-      <c r="E33" s="14"/>
-      <c r="F33" s="14"/>
-      <c r="G33" s="14"/>
-      <c r="H33" s="14"/>
-      <c r="I33" s="14" t="s">
-        <v>89</v>
-      </c>
-      <c r="J33" s="14" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="34" spans="1:10" ht="60">
-      <c r="A34" s="13" t="s">
-        <v>158</v>
-      </c>
-      <c r="B34" s="13" t="s">
-        <v>159</v>
-      </c>
-      <c r="C34" s="13" t="s">
-        <v>160</v>
-      </c>
-      <c r="D34" s="13" t="s">
+      <c r="E37" s="16"/>
+      <c r="F37" s="16"/>
+      <c r="G37" s="16"/>
+      <c r="H37" s="16"/>
+      <c r="I37" s="16"/>
+      <c r="J37" s="16"/>
+    </row>
+    <row r="38" spans="1:10" ht="120">
+      <c r="A38" s="15" t="s">
+        <v>168</v>
+      </c>
+      <c r="B38" s="15" t="s">
+        <v>169</v>
+      </c>
+      <c r="C38" s="15" t="s">
+        <v>170</v>
+      </c>
+      <c r="D38" s="15" t="s">
         <v>100</v>
       </c>
-      <c r="E34" s="14"/>
-      <c r="F34" s="14"/>
-      <c r="G34" s="14"/>
-      <c r="H34" s="14"/>
-      <c r="I34" s="14" t="s">
-        <v>178</v>
-      </c>
-      <c r="J34" s="14" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="35" spans="1:10" ht="30">
-      <c r="A35" s="13" t="s">
-        <v>161</v>
-      </c>
-      <c r="B35" s="13" t="s">
-        <v>162</v>
-      </c>
-      <c r="C35" s="13" t="s">
-        <v>143</v>
-      </c>
-      <c r="D35" s="13" t="s">
+      <c r="E38" s="16"/>
+      <c r="F38" s="16"/>
+      <c r="G38" s="16"/>
+      <c r="H38" s="16"/>
+      <c r="I38" s="16" t="s">
+        <v>175</v>
+      </c>
+      <c r="J38" s="16" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="39" spans="1:10" ht="75">
+      <c r="A39" s="15" t="s">
+        <v>171</v>
+      </c>
+      <c r="B39" s="15" t="s">
+        <v>172</v>
+      </c>
+      <c r="C39" s="15" t="s">
+        <v>173</v>
+      </c>
+      <c r="D39" s="15" t="s">
         <v>100</v>
       </c>
-      <c r="E35" s="14"/>
-      <c r="F35" s="14"/>
-      <c r="G35" s="14"/>
-      <c r="H35" s="14"/>
-      <c r="I35" s="14" t="s">
-        <v>89</v>
-      </c>
-      <c r="J35" s="14" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="36" spans="1:10" ht="60">
-      <c r="A36" s="13" t="s">
-        <v>165</v>
-      </c>
-      <c r="B36" s="13" t="s">
-        <v>166</v>
-      </c>
-      <c r="C36" s="13" t="s">
-        <v>160</v>
-      </c>
-      <c r="D36" s="13" t="s">
-        <v>100</v>
-      </c>
-      <c r="E36" s="14"/>
-      <c r="F36" s="14"/>
-      <c r="G36" s="14"/>
-      <c r="H36" s="14"/>
-      <c r="I36" s="14" t="s">
-        <v>178</v>
-      </c>
-      <c r="J36" s="14" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="37" spans="1:10" ht="60">
-      <c r="A37" s="13" t="s">
-        <v>167</v>
-      </c>
-      <c r="B37" s="13" t="s">
-        <v>168</v>
-      </c>
-      <c r="C37" s="13" t="s">
-        <v>169</v>
-      </c>
-      <c r="D37" s="13" t="s">
-        <v>100</v>
-      </c>
-      <c r="E37" s="14"/>
-      <c r="F37" s="14"/>
-      <c r="G37" s="14"/>
-      <c r="H37" s="14"/>
-      <c r="I37" s="14"/>
-      <c r="J37" s="14"/>
-    </row>
-    <row r="38" spans="1:10" ht="120">
-      <c r="A38" s="13" t="s">
-        <v>170</v>
-      </c>
-      <c r="B38" s="13" t="s">
-        <v>171</v>
-      </c>
-      <c r="C38" s="13" t="s">
-        <v>172</v>
-      </c>
-      <c r="D38" s="13" t="s">
-        <v>100</v>
-      </c>
-      <c r="E38" s="14"/>
-      <c r="F38" s="14"/>
-      <c r="G38" s="14"/>
-      <c r="H38" s="14"/>
-      <c r="I38" s="14" t="s">
-        <v>177</v>
-      </c>
-      <c r="J38" s="14" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="39" spans="1:10" ht="75">
-      <c r="A39" s="13" t="s">
-        <v>173</v>
-      </c>
-      <c r="B39" s="13" t="s">
-        <v>174</v>
-      </c>
-      <c r="C39" s="13" t="s">
-        <v>175</v>
-      </c>
-      <c r="D39" s="13" t="s">
-        <v>100</v>
-      </c>
-      <c r="E39" s="14"/>
-      <c r="F39" s="14"/>
-      <c r="G39" s="14"/>
-      <c r="H39" s="14"/>
-      <c r="I39" s="14"/>
-      <c r="J39" s="14"/>
+      <c r="E39" s="16"/>
+      <c r="F39" s="16"/>
+      <c r="G39" s="16"/>
+      <c r="H39" s="16"/>
+      <c r="I39" s="16"/>
+      <c r="J39" s="16"/>
     </row>
     <row r="40" spans="1:10" ht="39">
       <c r="A40" s="6" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B40" s="6" t="s">
         <v>30</v>
@@ -2674,7 +2681,7 @@
     </row>
     <row r="53" spans="1:11" ht="91">
       <c r="A53" s="6" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B53" s="6" t="s">
         <v>22</v>
@@ -2694,7 +2701,7 @@
     </row>
     <row r="54" spans="1:11" ht="39">
       <c r="A54" s="6" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B54" s="6" t="s">
         <v>43</v>
@@ -2714,7 +2721,7 @@
     </row>
     <row r="55" spans="1:11" ht="13">
       <c r="A55" s="6" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B55" s="6" t="s">
         <v>54</v>
@@ -2727,7 +2734,7 @@
         <v>3037556</v>
       </c>
       <c r="F55" s="6" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="G55" s="6">
         <v>8840</v>
@@ -2740,7 +2747,7 @@
     </row>
     <row r="56" spans="1:11" ht="13">
       <c r="A56" s="6" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B56" s="6" t="s">
         <v>55</v>
@@ -2779,7 +2786,7 @@
         <v>3027114</v>
       </c>
       <c r="F57" s="6" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="G57" s="6">
         <v>8840</v>
@@ -2813,7 +2820,7 @@
       <c r="G58" s="10"/>
       <c r="H58" s="10"/>
       <c r="I58" s="12" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="J58" s="12" t="s">
         <v>102</v>
@@ -2828,4 +2835,10 @@
     <oddFooter>&amp;L_x000D_&amp;1#&amp;"Calibri"&amp;10&amp;K000000 INTERNAL</oddFooter>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{3ca48ea3-8c75-4d36-b64f-70604b11fd22}" enabled="1" method="Standard" siteId="{3ac94b33-9135-4821-9502-eafda6592a35}" contentBits="0" removed="0"/>
+</clbl:labelList>
 </file>
</xml_diff>